<commit_message>
Alternate added for header in client bom
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/FLST_Client BOM.xlsx
+++ b/Deliverables/BOM/FLST_Client BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\flst\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\flst\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="161">
   <si>
     <t>Description</t>
   </si>
@@ -503,7 +503,10 @@
     <t>SOP-4</t>
   </si>
   <si>
-    <t>Quotation Required</t>
+    <t>C390678</t>
+  </si>
+  <si>
+    <t>210-91-02GB01</t>
   </si>
 </sst>
 </file>
@@ -514,7 +517,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -537,12 +540,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -574,21 +571,36 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF333333"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -604,12 +616,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -729,90 +735,102 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1096,7 +1114,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
@@ -1117,25 +1135,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="28"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="17"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1194,31 +1212,31 @@
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="14" t="s">
         <v>147</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="27" t="s">
         <v>108</v>
       </c>
-      <c r="I3" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J3" s="9" t="s">
+      <c r="I3" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J3" s="8" t="s">
         <v>4</v>
       </c>
       <c r="K3" s="5">
@@ -1231,13 +1249,13 @@
       <c r="M3" s="5">
         <v>7</v>
       </c>
-      <c r="N3" s="10" t="s">
+      <c r="N3" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O3" s="17">
+      <c r="O3" s="28">
         <v>1.3327</v>
       </c>
-      <c r="P3" s="18">
+      <c r="P3" s="11">
         <f>O3*M3</f>
         <v>9.3289000000000009</v>
       </c>
@@ -1248,29 +1266,29 @@
         <f>A3+1</f>
         <v>2</v>
       </c>
-      <c r="B4" s="24"/>
+      <c r="B4" s="14"/>
       <c r="C4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="I4" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J4" s="9" t="s">
+      <c r="I4" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J4" s="8" t="s">
         <v>9</v>
       </c>
       <c r="K4" s="5">
@@ -1283,13 +1301,13 @@
       <c r="M4" s="5">
         <v>7</v>
       </c>
-      <c r="N4" s="10" t="s">
+      <c r="N4" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O4" s="17">
+      <c r="O4" s="28">
         <v>0.39140000000000003</v>
       </c>
-      <c r="P4" s="18">
+      <c r="P4" s="11">
         <f t="shared" ref="P4:P25" si="1">O4*M4</f>
         <v>2.7398000000000002</v>
       </c>
@@ -1300,29 +1318,29 @@
         <f t="shared" ref="A5:A25" si="2">A4+1</f>
         <v>3</v>
       </c>
-      <c r="B5" s="24"/>
+      <c r="B5" s="14"/>
       <c r="C5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="I5" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J5" s="9" t="s">
+      <c r="I5" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>13</v>
       </c>
       <c r="K5" s="5">
@@ -1335,13 +1353,13 @@
       <c r="M5" s="5">
         <v>100</v>
       </c>
-      <c r="N5" s="10" t="s">
+      <c r="N5" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O5" s="17">
+      <c r="O5" s="28">
         <v>3.3E-3</v>
       </c>
-      <c r="P5" s="18">
+      <c r="P5" s="11">
         <f t="shared" si="1"/>
         <v>0.33</v>
       </c>
@@ -1352,29 +1370,29 @@
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="B6" s="24"/>
+      <c r="B6" s="14"/>
       <c r="C6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="I6" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J6" s="9" t="s">
+      <c r="I6" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="K6" s="5">
@@ -1387,13 +1405,13 @@
       <c r="M6" s="5">
         <v>100</v>
       </c>
-      <c r="N6" s="10" t="s">
+      <c r="N6" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O6" s="17">
+      <c r="O6" s="28">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="P6" s="18">
+      <c r="P6" s="11">
         <f t="shared" si="1"/>
         <v>0.33999999999999997</v>
       </c>
@@ -1404,29 +1422,29 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="B7" s="24"/>
+      <c r="B7" s="14"/>
       <c r="C7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="I7" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J7" s="9" t="s">
+      <c r="I7" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J7" s="8" t="s">
         <v>22</v>
       </c>
       <c r="K7" s="5">
@@ -1439,13 +1457,13 @@
       <c r="M7" s="5">
         <v>50</v>
       </c>
-      <c r="N7" s="10" t="s">
+      <c r="N7" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O7" s="17">
+      <c r="O7" s="28">
         <v>7.1000000000000004E-3</v>
       </c>
-      <c r="P7" s="18">
+      <c r="P7" s="11">
         <f t="shared" si="1"/>
         <v>0.35500000000000004</v>
       </c>
@@ -1456,31 +1474,31 @@
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="13" t="s">
         <v>148</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="I8" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J8" s="12" t="s">
+      <c r="I8" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J8" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K8" s="5">
@@ -1493,13 +1511,13 @@
       <c r="M8" s="5">
         <v>10</v>
       </c>
-      <c r="N8" s="10" t="s">
+      <c r="N8" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O8" s="17">
+      <c r="O8" s="28">
         <v>4.0599999999999997E-2</v>
       </c>
-      <c r="P8" s="18">
+      <c r="P8" s="11">
         <f t="shared" si="1"/>
         <v>0.40599999999999997</v>
       </c>
@@ -1510,31 +1528,31 @@
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="13" t="s">
         <v>149</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="I9" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J9" s="12" t="s">
+      <c r="I9" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J9" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K9" s="5">
@@ -1547,13 +1565,13 @@
       <c r="M9" s="5">
         <v>22</v>
       </c>
-      <c r="N9" s="10" t="s">
+      <c r="N9" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O9" s="17">
+      <c r="O9" s="28">
         <v>0.31</v>
       </c>
-      <c r="P9" s="18">
+      <c r="P9" s="11">
         <f t="shared" si="1"/>
         <v>6.82</v>
       </c>
@@ -1564,31 +1582,31 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="14" t="s">
         <v>150</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="I10" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J10" s="9" t="s">
+      <c r="I10" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>32</v>
       </c>
       <c r="K10" s="5">
@@ -1601,13 +1619,13 @@
       <c r="M10" s="5">
         <v>7</v>
       </c>
-      <c r="N10" s="10" t="s">
+      <c r="N10" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O10" s="17">
+      <c r="O10" s="28">
         <v>0.44369999999999998</v>
       </c>
-      <c r="P10" s="18">
+      <c r="P10" s="11">
         <f t="shared" si="1"/>
         <v>3.1059000000000001</v>
       </c>
@@ -1618,29 +1636,29 @@
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="B11" s="24"/>
+      <c r="B11" s="14"/>
       <c r="C11" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="8" t="s">
         <v>36</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="H11" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="I11" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J11" s="12" t="s">
+      <c r="I11" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J11" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K11" s="5">
@@ -1653,13 +1671,13 @@
       <c r="M11" s="5">
         <v>50</v>
       </c>
-      <c r="N11" s="10" t="s">
+      <c r="N11" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O11" s="17">
+      <c r="O11" s="28">
         <v>1.5599999999999999E-2</v>
       </c>
-      <c r="P11" s="18">
+      <c r="P11" s="11">
         <f t="shared" si="1"/>
         <v>0.77999999999999992</v>
       </c>
@@ -1670,31 +1688,31 @@
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="14" t="s">
         <v>151</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="27" t="s">
         <v>125</v>
       </c>
-      <c r="I12" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J12" s="9" t="s">
+      <c r="I12" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J12" s="8" t="s">
         <v>47</v>
       </c>
       <c r="K12" s="5">
@@ -1707,13 +1725,13 @@
       <c r="M12" s="5">
         <v>50</v>
       </c>
-      <c r="N12" s="10" t="s">
+      <c r="N12" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O12" s="17">
+      <c r="O12" s="28">
         <v>4.3E-3</v>
       </c>
-      <c r="P12" s="18">
+      <c r="P12" s="11">
         <f t="shared" si="1"/>
         <v>0.215</v>
       </c>
@@ -1724,29 +1742,29 @@
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="B13" s="24"/>
+      <c r="B13" s="14"/>
       <c r="C13" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="8" t="s">
         <v>55</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="29" t="s">
         <v>126</v>
       </c>
-      <c r="I13" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J13" s="9" t="s">
+      <c r="I13" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J13" s="8" t="s">
         <v>52</v>
       </c>
       <c r="K13" s="5">
@@ -1759,13 +1777,13 @@
       <c r="M13" s="5">
         <v>100</v>
       </c>
-      <c r="N13" s="10" t="s">
+      <c r="N13" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O13" s="17">
+      <c r="O13" s="28">
         <v>1.5E-3</v>
       </c>
-      <c r="P13" s="18">
+      <c r="P13" s="11">
         <f t="shared" si="1"/>
         <v>0.15</v>
       </c>
@@ -1776,29 +1794,29 @@
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="B14" s="24"/>
+      <c r="B14" s="14"/>
       <c r="C14" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>60</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="H14" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="I14" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J14" s="9" t="s">
+      <c r="I14" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J14" s="8" t="s">
         <v>56</v>
       </c>
       <c r="K14" s="5">
@@ -1811,13 +1829,13 @@
       <c r="M14" s="5">
         <v>100</v>
       </c>
-      <c r="N14" s="10" t="s">
+      <c r="N14" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O14" s="17">
+      <c r="O14" s="28">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="P14" s="18">
+      <c r="P14" s="11">
         <f t="shared" si="1"/>
         <v>0.12</v>
       </c>
@@ -1828,29 +1846,29 @@
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="B15" s="24"/>
+      <c r="B15" s="14"/>
       <c r="C15" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="H15" s="29" t="s">
         <v>128</v>
       </c>
-      <c r="I15" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J15" s="9" t="s">
+      <c r="I15" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J15" s="8" t="s">
         <v>61</v>
       </c>
       <c r="K15" s="5">
@@ -1863,13 +1881,13 @@
       <c r="M15" s="5">
         <v>100</v>
       </c>
-      <c r="N15" s="10" t="s">
+      <c r="N15" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O15" s="17">
+      <c r="O15" s="28">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="P15" s="18">
+      <c r="P15" s="11">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
@@ -1880,29 +1898,29 @@
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="B16" s="24"/>
+      <c r="B16" s="14"/>
       <c r="C16" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="G16" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="29" t="s">
         <v>129</v>
       </c>
-      <c r="I16" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J16" s="9" t="s">
+      <c r="I16" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J16" s="8" t="s">
         <v>65</v>
       </c>
       <c r="K16" s="5">
@@ -1915,46 +1933,46 @@
       <c r="M16" s="5">
         <v>50</v>
       </c>
-      <c r="N16" s="10" t="s">
+      <c r="N16" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O16" s="17">
+      <c r="O16" s="28">
         <v>1.52E-2</v>
       </c>
-      <c r="P16" s="18">
+      <c r="P16" s="11">
         <f t="shared" si="1"/>
         <v>0.76</v>
       </c>
       <c r="Q16" s="5"/>
     </row>
-    <row r="17" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="B17" s="24"/>
+      <c r="B17" s="14"/>
       <c r="C17" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="8" t="s">
         <v>72</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="H17" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="I17" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J17" s="9" t="s">
+      <c r="I17" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J17" s="8" t="s">
         <v>69</v>
       </c>
       <c r="K17" s="5">
@@ -1967,46 +1985,46 @@
       <c r="M17" s="5">
         <v>100</v>
       </c>
-      <c r="N17" s="10" t="s">
+      <c r="N17" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O17" s="17">
+      <c r="O17" s="28">
         <v>1.5E-3</v>
       </c>
-      <c r="P17" s="18">
+      <c r="P17" s="11">
         <f t="shared" si="1"/>
         <v>0.15</v>
       </c>
       <c r="Q17" s="5"/>
     </row>
-    <row r="18" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="B18" s="24"/>
+      <c r="B18" s="14"/>
       <c r="C18" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="G18" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="I18" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J18" s="9" t="s">
+      <c r="I18" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J18" s="8" t="s">
         <v>73</v>
       </c>
       <c r="K18" s="5">
@@ -2019,48 +2037,48 @@
       <c r="M18" s="5">
         <v>100</v>
       </c>
-      <c r="N18" s="10" t="s">
+      <c r="N18" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O18" s="17">
+      <c r="O18" s="28">
         <v>1.4E-3</v>
       </c>
-      <c r="P18" s="18">
+      <c r="P18" s="11">
         <f t="shared" si="1"/>
         <v>0.13999999999999999</v>
       </c>
       <c r="Q18" s="5"/>
     </row>
-    <row r="19" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="13" t="s">
         <v>152</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="G19" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="H19" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="I19" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J19" s="12" t="s">
+      <c r="I19" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J19" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K19" s="5">
@@ -2073,48 +2091,48 @@
       <c r="M19" s="5">
         <v>10</v>
       </c>
-      <c r="N19" s="10" t="s">
+      <c r="N19" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O19" s="17">
+      <c r="O19" s="28">
         <v>5.9499999999999997E-2</v>
       </c>
-      <c r="P19" s="18">
+      <c r="P19" s="11">
         <f t="shared" si="1"/>
         <v>0.59499999999999997</v>
       </c>
       <c r="Q19" s="5"/>
     </row>
-    <row r="20" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="14" t="s">
         <v>156</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="H20" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="I20" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J20" s="12" t="s">
+      <c r="I20" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J20" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K20" s="5">
@@ -2127,46 +2145,46 @@
       <c r="M20" s="5">
         <v>7</v>
       </c>
-      <c r="N20" s="10" t="s">
+      <c r="N20" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O20" s="17">
+      <c r="O20" s="28">
         <v>0.4869</v>
       </c>
-      <c r="P20" s="18">
+      <c r="P20" s="11">
         <f t="shared" si="1"/>
         <v>3.4083000000000001</v>
       </c>
       <c r="Q20" s="5"/>
     </row>
-    <row r="21" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="B21" s="24"/>
+      <c r="B21" s="14"/>
       <c r="C21" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="8" t="s">
         <v>84</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="H21" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="I21" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J21" s="12" t="s">
+      <c r="I21" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J21" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K21" s="5">
@@ -2179,46 +2197,46 @@
       <c r="M21" s="5">
         <v>7</v>
       </c>
-      <c r="N21" s="10" t="s">
+      <c r="N21" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O21" s="17">
+      <c r="O21" s="28">
         <v>1.8827</v>
       </c>
-      <c r="P21" s="18">
+      <c r="P21" s="11">
         <f t="shared" si="1"/>
         <v>13.178900000000001</v>
       </c>
       <c r="Q21" s="5"/>
     </row>
-    <row r="22" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="B22" s="24"/>
+      <c r="B22" s="14"/>
       <c r="C22" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="G22" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="H22" s="27" t="s">
         <v>140</v>
       </c>
-      <c r="I22" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J22" s="12" t="s">
+      <c r="I22" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J22" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K22" s="5">
@@ -2231,46 +2249,46 @@
       <c r="M22" s="5">
         <v>7</v>
       </c>
-      <c r="N22" s="10" t="s">
+      <c r="N22" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O22" s="17">
+      <c r="O22" s="28">
         <v>0.95220000000000005</v>
       </c>
-      <c r="P22" s="18">
+      <c r="P22" s="11">
         <f t="shared" si="1"/>
         <v>6.6654</v>
       </c>
       <c r="Q22" s="5"/>
     </row>
-    <row r="23" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="B23" s="24"/>
+      <c r="B23" s="14"/>
       <c r="C23" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="G23" s="10" t="s">
+      <c r="G23" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="H23" s="11" t="s">
+      <c r="H23" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="I23" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J23" s="12" t="s">
+      <c r="I23" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J23" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K23" s="5">
@@ -2283,48 +2301,48 @@
       <c r="M23" s="5">
         <v>7</v>
       </c>
-      <c r="N23" s="10" t="s">
+      <c r="N23" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O23" s="17">
+      <c r="O23" s="28">
         <v>0.54279999999999995</v>
       </c>
-      <c r="P23" s="18">
+      <c r="P23" s="11">
         <f t="shared" si="1"/>
         <v>3.7995999999999999</v>
       </c>
       <c r="Q23" s="5"/>
     </row>
-    <row r="24" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <f t="shared" si="2"/>
         <v>22</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="14" t="s">
         <v>153</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G24" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="H24" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="I24" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J24" s="12" t="s">
+      <c r="I24" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="J24" s="10" t="s">
         <v>146</v>
       </c>
       <c r="K24" s="5">
@@ -2337,88 +2355,111 @@
       <c r="M24" s="5">
         <v>20</v>
       </c>
-      <c r="N24" s="10" t="s">
+      <c r="N24" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O24" s="17">
+      <c r="O24" s="28">
         <v>3.1399999999999997E-2</v>
       </c>
-      <c r="P24" s="18">
+      <c r="P24" s="11">
         <f t="shared" si="1"/>
         <v>0.62799999999999989</v>
       </c>
       <c r="Q24" s="5"/>
     </row>
-    <row r="25" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <f t="shared" si="2"/>
         <v>23</v>
       </c>
-      <c r="B25" s="24"/>
-      <c r="C25" s="13" t="s">
+      <c r="B25" s="14"/>
+      <c r="C25" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="D25" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="E25" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="F25" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="G25" s="15" t="s">
+      <c r="G25" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="H25" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="J25" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="K25" s="16">
+      <c r="H25" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="I25" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="J25" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="K25" s="21">
         <v>10</v>
       </c>
-      <c r="L25" s="16">
+      <c r="L25" s="21">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="21">
+      <c r="M25" s="21">
+        <v>100</v>
+      </c>
+      <c r="N25" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="O25" s="26">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="P25" s="22">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="23" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="K26" s="25" t="s">
+        <v>0.89999999999999991</v>
+      </c>
+      <c r="Q25" s="23"/>
+      <c r="R25" s="24"/>
+    </row>
+    <row r="26" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="L26" s="25"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="25"/>
-      <c r="P26" s="19">
+      <c r="L26" s="33"/>
+      <c r="M26" s="33"/>
+      <c r="N26" s="33"/>
+      <c r="O26" s="31"/>
+      <c r="P26" s="12">
         <f>SUM(P3:P25)</f>
-        <v>54.175800000000002</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="K27" s="25" t="s">
+        <v>55.075800000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="31"/>
+      <c r="I27" s="31"/>
+      <c r="J27" s="31"/>
+      <c r="K27" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="L27" s="25"/>
-      <c r="M27" s="25"/>
-      <c r="N27" s="25"/>
-      <c r="P27" s="20">
+      <c r="L27" s="33"/>
+      <c r="M27" s="33"/>
+      <c r="N27" s="33"/>
+      <c r="O27" s="31"/>
+      <c r="P27" s="34">
         <f>P26/5</f>
-        <v>10.83516</v>
+        <v>11.01516</v>
       </c>
     </row>
   </sheetData>
@@ -2518,9 +2559,10 @@
     <hyperlink ref="G24" r:id="rId43" display="https://lcsc.com/brand-detail/12130.html"/>
     <hyperlink ref="N24" r:id="rId44"/>
     <hyperlink ref="G25" r:id="rId45" display="https://www.chip1stop.com/USA/en/maker/wurth"/>
+    <hyperlink ref="N25" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId46"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId47"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
Total price divided by 5
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/FLST_Client BOM.xlsx
+++ b/Deliverables/BOM/FLST_Client BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\flst\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\flst\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8191372C-7AD2-494A-AEC2-D00A87B0D426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17010" yWindow="240" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17010" yWindow="240" windowWidth="11790" windowHeight="15360"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -533,7 +532,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1212,7 +1211,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1343,6 +1341,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1678,7 +1677,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Q34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1711,9 +1710,9 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="89"/>
+      <c r="J1" s="87"/>
+      <c r="K1" s="87"/>
+      <c r="L1" s="88"/>
     </row>
     <row r="2" spans="1:17" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1731,12 +1730,12 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="82"/>
-      <c r="M2" s="82"/>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
-      <c r="P2" s="82"/>
-      <c r="Q2" s="83"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="81"/>
+      <c r="N2" s="81"/>
+      <c r="O2" s="81"/>
+      <c r="P2" s="81"/>
+      <c r="Q2" s="82"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -1759,7 +1758,7 @@
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
-      <c r="Q3" s="84"/>
+      <c r="Q3" s="83"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1782,7 +1781,7 @@
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
-      <c r="Q4" s="85"/>
+      <c r="Q4" s="84"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1805,7 +1804,7 @@
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
-      <c r="Q5" s="85"/>
+      <c r="Q5" s="84"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1824,7 +1823,7 @@
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
-      <c r="Q6" s="85"/>
+      <c r="Q6" s="84"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1843,7 +1842,7 @@
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
-      <c r="Q7" s="85"/>
+      <c r="Q7" s="84"/>
     </row>
     <row r="8" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1862,7 +1861,7 @@
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
-      <c r="Q8" s="85"/>
+      <c r="Q8" s="84"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1878,19 +1877,19 @@
       <c r="E9" s="39" t="s">
         <v>58</v>
       </c>
-      <c r="F9" s="48" t="s">
+      <c r="F9" s="47" t="s">
         <v>75</v>
       </c>
       <c r="G9" s="39" t="s">
         <v>123</v>
       </c>
-      <c r="H9" s="48" t="s">
+      <c r="H9" s="47" t="s">
         <v>89</v>
       </c>
       <c r="I9" s="39" t="s">
         <v>124</v>
       </c>
-      <c r="J9" s="48" t="s">
+      <c r="J9" s="47" t="s">
         <v>106</v>
       </c>
       <c r="K9" s="39" t="s">
@@ -1899,13 +1898,13 @@
       <c r="L9" s="39" t="s">
         <v>126</v>
       </c>
-      <c r="M9" s="48" t="s">
+      <c r="M9" s="47" t="s">
         <v>127</v>
       </c>
       <c r="N9" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="O9" s="48" t="s">
+      <c r="O9" s="47" t="s">
         <v>129</v>
       </c>
       <c r="P9" s="39" t="s">
@@ -1921,47 +1920,47 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="68" t="s">
+      <c r="C10" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="68" t="s">
+      <c r="D10" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="68" t="s">
+      <c r="E10" s="67" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="69" t="s">
+      <c r="F10" s="68" t="s">
         <v>76</v>
       </c>
-      <c r="G10" s="68" t="s">
+      <c r="G10" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H10" s="69" t="s">
+      <c r="H10" s="68" t="s">
         <v>90</v>
       </c>
-      <c r="I10" s="68" t="s">
+      <c r="I10" s="67" t="s">
         <v>131</v>
       </c>
-      <c r="J10" s="69" t="s">
+      <c r="J10" s="68" t="s">
         <v>107</v>
       </c>
-      <c r="K10" s="68">
+      <c r="K10" s="67">
         <v>1</v>
       </c>
-      <c r="L10" s="68">
+      <c r="L10" s="67">
         <f>K10*5</f>
         <v>5</v>
       </c>
-      <c r="M10" s="69">
+      <c r="M10" s="68">
         <v>7</v>
       </c>
-      <c r="N10" s="56" t="s">
+      <c r="N10" s="55" t="s">
         <v>136</v>
       </c>
-      <c r="O10" s="49">
+      <c r="O10" s="48">
         <v>1.3327</v>
       </c>
-      <c r="P10" s="75">
+      <c r="P10" s="74">
         <f>O10*M10</f>
         <v>9.3289000000000009</v>
       </c>
@@ -1973,47 +1972,47 @@
         <f t="shared" ref="B11:B31" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="70" t="s">
+      <c r="C11" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="70" t="s">
+      <c r="D11" s="69" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="70" t="s">
+      <c r="E11" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="F11" s="71" t="s">
+      <c r="F11" s="70" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="70" t="s">
+      <c r="G11" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H11" s="71" t="s">
+      <c r="H11" s="70" t="s">
         <v>91</v>
       </c>
-      <c r="I11" s="70" t="s">
+      <c r="I11" s="69" t="s">
         <v>132</v>
       </c>
-      <c r="J11" s="71" t="s">
+      <c r="J11" s="70" t="s">
         <v>108</v>
       </c>
-      <c r="K11" s="70">
+      <c r="K11" s="69">
         <v>1</v>
       </c>
-      <c r="L11" s="70">
+      <c r="L11" s="69">
         <f t="shared" ref="L11:L32" si="1">K11*5</f>
         <v>5</v>
       </c>
-      <c r="M11" s="71">
+      <c r="M11" s="70">
         <v>7</v>
       </c>
-      <c r="N11" s="57" t="s">
+      <c r="N11" s="56" t="s">
         <v>136</v>
       </c>
-      <c r="O11" s="50">
+      <c r="O11" s="49">
         <v>0.39140000000000003</v>
       </c>
-      <c r="P11" s="76">
+      <c r="P11" s="75">
         <f t="shared" ref="P11:P32" si="2">O11*M11</f>
         <v>2.7398000000000002</v>
       </c>
@@ -2025,47 +2024,47 @@
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="68" t="s">
+      <c r="C12" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="68" t="s">
+      <c r="D12" s="67" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="68" t="s">
+      <c r="E12" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="69" t="s">
+      <c r="F12" s="68" t="s">
         <v>77</v>
       </c>
-      <c r="G12" s="68" t="s">
+      <c r="G12" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H12" s="69" t="s">
+      <c r="H12" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="I12" s="68" t="s">
+      <c r="I12" s="67" t="s">
         <v>133</v>
       </c>
-      <c r="J12" s="69" t="s">
+      <c r="J12" s="68" t="s">
         <v>109</v>
       </c>
-      <c r="K12" s="68">
+      <c r="K12" s="67">
         <v>1</v>
       </c>
-      <c r="L12" s="68">
+      <c r="L12" s="67">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M12" s="69">
+      <c r="M12" s="68">
         <v>100</v>
       </c>
-      <c r="N12" s="58" t="s">
+      <c r="N12" s="57" t="s">
         <v>136</v>
       </c>
-      <c r="O12" s="51">
+      <c r="O12" s="50">
         <v>3.3E-3</v>
       </c>
-      <c r="P12" s="75">
+      <c r="P12" s="74">
         <f t="shared" si="2"/>
         <v>0.33</v>
       </c>
@@ -2077,47 +2076,47 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="70" t="s">
+      <c r="C13" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="70" t="s">
+      <c r="D13" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="70" t="s">
+      <c r="E13" s="69" t="s">
         <v>61</v>
       </c>
-      <c r="F13" s="71" t="s">
+      <c r="F13" s="70" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="70" t="s">
+      <c r="G13" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H13" s="71" t="s">
+      <c r="H13" s="70" t="s">
         <v>92</v>
       </c>
-      <c r="I13" s="70" t="s">
+      <c r="I13" s="69" t="s">
         <v>134</v>
       </c>
-      <c r="J13" s="71" t="s">
+      <c r="J13" s="70" t="s">
         <v>110</v>
       </c>
-      <c r="K13" s="70">
+      <c r="K13" s="69">
         <v>2</v>
       </c>
-      <c r="L13" s="70">
+      <c r="L13" s="69">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="M13" s="71">
+      <c r="M13" s="70">
         <v>100</v>
       </c>
-      <c r="N13" s="59" t="s">
+      <c r="N13" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="O13" s="50">
+      <c r="O13" s="49">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="P13" s="76">
+      <c r="P13" s="75">
         <f t="shared" si="2"/>
         <v>0.33999999999999997</v>
       </c>
@@ -2129,47 +2128,47 @@
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="68" t="s">
+      <c r="C14" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="68" t="s">
+      <c r="D14" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="68" t="s">
+      <c r="E14" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="69" t="s">
+      <c r="F14" s="68" t="s">
         <v>79</v>
       </c>
-      <c r="G14" s="68" t="s">
+      <c r="G14" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H14" s="69" t="s">
+      <c r="H14" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="I14" s="68" t="s">
+      <c r="I14" s="67" t="s">
         <v>135</v>
       </c>
-      <c r="J14" s="69" t="s">
+      <c r="J14" s="68" t="s">
         <v>111</v>
       </c>
-      <c r="K14" s="68">
+      <c r="K14" s="67">
         <v>1</v>
       </c>
-      <c r="L14" s="68">
+      <c r="L14" s="67">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M14" s="69">
+      <c r="M14" s="68">
         <v>50</v>
       </c>
-      <c r="N14" s="58" t="s">
+      <c r="N14" s="57" t="s">
         <v>136</v>
       </c>
-      <c r="O14" s="51">
+      <c r="O14" s="50">
         <v>7.1000000000000004E-3</v>
       </c>
-      <c r="P14" s="75">
+      <c r="P14" s="74">
         <f t="shared" si="2"/>
         <v>0.35500000000000004</v>
       </c>
@@ -2181,47 +2180,47 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="70" t="s">
+      <c r="C15" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="70" t="s">
+      <c r="D15" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="70" t="s">
+      <c r="E15" s="69" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="71" t="s">
+      <c r="F15" s="70" t="s">
         <v>112</v>
       </c>
-      <c r="G15" s="70" t="s">
+      <c r="G15" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H15" s="71" t="s">
+      <c r="H15" s="70" t="s">
         <v>93</v>
       </c>
-      <c r="I15" s="70" t="s">
+      <c r="I15" s="69" t="s">
         <v>138</v>
       </c>
-      <c r="J15" s="71" t="s">
+      <c r="J15" s="70" t="s">
         <v>139</v>
       </c>
-      <c r="K15" s="70">
+      <c r="K15" s="69">
         <v>1</v>
       </c>
-      <c r="L15" s="70">
+      <c r="L15" s="69">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M15" s="71">
+      <c r="M15" s="70">
         <v>10</v>
       </c>
-      <c r="N15" s="59" t="s">
+      <c r="N15" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="O15" s="50">
+      <c r="O15" s="49">
         <v>4.0599999999999997E-2</v>
       </c>
-      <c r="P15" s="76">
+      <c r="P15" s="75">
         <f t="shared" si="2"/>
         <v>0.40599999999999997</v>
       </c>
@@ -2233,47 +2232,47 @@
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="68" t="s">
+      <c r="C16" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="68" t="s">
+      <c r="D16" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="68" t="s">
+      <c r="E16" s="67" t="s">
         <v>63</v>
       </c>
-      <c r="F16" s="69" t="s">
+      <c r="F16" s="68" t="s">
         <v>113</v>
       </c>
-      <c r="G16" s="68" t="s">
+      <c r="G16" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H16" s="69" t="s">
+      <c r="H16" s="68" t="s">
         <v>94</v>
       </c>
-      <c r="I16" s="68" t="s">
+      <c r="I16" s="67" t="s">
         <v>140</v>
       </c>
-      <c r="J16" s="69" t="s">
+      <c r="J16" s="68" t="s">
         <v>155</v>
       </c>
-      <c r="K16" s="68">
+      <c r="K16" s="67">
         <v>1</v>
       </c>
-      <c r="L16" s="68">
+      <c r="L16" s="67">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M16" s="69">
+      <c r="M16" s="68">
         <v>20</v>
       </c>
-      <c r="N16" s="60" t="s">
+      <c r="N16" s="59" t="s">
         <v>136</v>
       </c>
-      <c r="O16" s="52">
+      <c r="O16" s="51">
         <v>3.1399999999999997E-2</v>
       </c>
-      <c r="P16" s="75">
+      <c r="P16" s="74">
         <f t="shared" si="2"/>
         <v>0.62799999999999989</v>
       </c>
@@ -2285,47 +2284,47 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="70" t="s">
+      <c r="C17" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="70" t="s">
+      <c r="D17" s="69" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="70" t="s">
+      <c r="E17" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="F17" s="71" t="s">
+      <c r="F17" s="70" t="s">
         <v>64</v>
       </c>
-      <c r="G17" s="70" t="s">
+      <c r="G17" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H17" s="71" t="s">
+      <c r="H17" s="70" t="s">
         <v>95</v>
       </c>
-      <c r="I17" s="70" t="s">
+      <c r="I17" s="69" t="s">
         <v>141</v>
       </c>
-      <c r="J17" s="71" t="s">
+      <c r="J17" s="70" t="s">
         <v>114</v>
       </c>
-      <c r="K17" s="70">
+      <c r="K17" s="69">
         <v>1</v>
       </c>
-      <c r="L17" s="70">
+      <c r="L17" s="69">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M17" s="71">
+      <c r="M17" s="70">
         <v>7</v>
       </c>
-      <c r="N17" s="61" t="s">
+      <c r="N17" s="60" t="s">
         <v>136</v>
       </c>
-      <c r="O17" s="53">
+      <c r="O17" s="52">
         <v>0.44369999999999998</v>
       </c>
-      <c r="P17" s="76">
+      <c r="P17" s="75">
         <f t="shared" si="2"/>
         <v>3.1059000000000001</v>
       </c>
@@ -2337,47 +2336,47 @@
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="68" t="s">
+      <c r="C18" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="68" t="s">
+      <c r="D18" s="67" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="68" t="s">
+      <c r="E18" s="67" t="s">
         <v>65</v>
       </c>
-      <c r="F18" s="69" t="s">
+      <c r="F18" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="G18" s="68" t="s">
+      <c r="G18" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H18" s="69" t="s">
+      <c r="H18" s="68" t="s">
         <v>95</v>
       </c>
-      <c r="I18" s="68" t="s">
+      <c r="I18" s="67" t="s">
         <v>142</v>
       </c>
-      <c r="J18" s="69" t="s">
+      <c r="J18" s="68" t="s">
         <v>155</v>
       </c>
-      <c r="K18" s="68">
+      <c r="K18" s="67">
         <v>1</v>
       </c>
-      <c r="L18" s="68">
+      <c r="L18" s="67">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M18" s="69">
+      <c r="M18" s="68">
         <v>50</v>
       </c>
-      <c r="N18" s="62" t="s">
+      <c r="N18" s="61" t="s">
         <v>136</v>
       </c>
-      <c r="O18" s="51">
+      <c r="O18" s="50">
         <v>1.5599999999999999E-2</v>
       </c>
-      <c r="P18" s="75">
+      <c r="P18" s="74">
         <f t="shared" si="2"/>
         <v>0.77999999999999992</v>
       </c>
@@ -2389,47 +2388,47 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="70" t="s">
+      <c r="C19" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="70" t="s">
+      <c r="D19" s="69" t="s">
         <v>44</v>
       </c>
-      <c r="E19" s="70" t="s">
+      <c r="E19" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="F19" s="71">
+      <c r="F19" s="70">
         <v>61300211121</v>
       </c>
-      <c r="G19" s="70" t="s">
+      <c r="G19" s="69" t="s">
         <v>144</v>
       </c>
-      <c r="H19" s="71" t="s">
+      <c r="H19" s="70" t="s">
         <v>96</v>
       </c>
-      <c r="I19" s="70" t="s">
+      <c r="I19" s="69" t="s">
         <v>143</v>
       </c>
-      <c r="J19" s="71" t="s">
+      <c r="J19" s="70" t="s">
         <v>155</v>
       </c>
-      <c r="K19" s="70">
+      <c r="K19" s="69">
         <v>10</v>
       </c>
-      <c r="L19" s="70">
+      <c r="L19" s="69">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="M19" s="71">
+      <c r="M19" s="70">
         <v>100</v>
       </c>
-      <c r="N19" s="63" t="s">
+      <c r="N19" s="62" t="s">
         <v>136</v>
       </c>
       <c r="O19" s="40">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="P19" s="76">
+      <c r="P19" s="75">
         <f t="shared" si="2"/>
         <v>0.89999999999999991</v>
       </c>
@@ -2441,45 +2440,45 @@
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="68" t="s">
+      <c r="C20" s="67" t="s">
         <v>21</v>
       </c>
-      <c r="D20" s="68" t="s">
+      <c r="D20" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="68" t="s">
+      <c r="E20" s="67" t="s">
         <v>67</v>
       </c>
-      <c r="F20" s="69" t="s">
+      <c r="F20" s="68" t="s">
         <v>81</v>
       </c>
-      <c r="G20" s="68" t="s">
+      <c r="G20" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H20" s="69" t="s">
+      <c r="H20" s="68" t="s">
         <v>97</v>
       </c>
-      <c r="I20" s="68" t="s">
+      <c r="I20" s="67" t="s">
         <v>145</v>
       </c>
-      <c r="J20" s="69"/>
-      <c r="K20" s="68">
+      <c r="J20" s="68"/>
+      <c r="K20" s="67">
         <v>4</v>
       </c>
-      <c r="L20" s="68">
+      <c r="L20" s="67">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="M20" s="69">
+      <c r="M20" s="68">
         <v>22</v>
       </c>
-      <c r="N20" s="58" t="s">
+      <c r="N20" s="57" t="s">
         <v>136</v>
       </c>
-      <c r="O20" s="51">
+      <c r="O20" s="50">
         <v>0.3644</v>
       </c>
-      <c r="P20" s="75">
+      <c r="P20" s="74">
         <f t="shared" si="2"/>
         <v>8.0167999999999999</v>
       </c>
@@ -2491,47 +2490,47 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="70" t="s">
+      <c r="C21" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="D21" s="70" t="s">
+      <c r="D21" s="69" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="70" t="s">
+      <c r="E21" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="F21" s="71" t="s">
+      <c r="F21" s="70" t="s">
         <v>146</v>
       </c>
-      <c r="G21" s="70" t="s">
+      <c r="G21" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H21" s="71" t="s">
+      <c r="H21" s="70" t="s">
         <v>98</v>
       </c>
-      <c r="I21" s="70" t="s">
+      <c r="I21" s="69" t="s">
         <v>147</v>
       </c>
-      <c r="J21" s="71" t="s">
+      <c r="J21" s="70" t="s">
         <v>115</v>
       </c>
-      <c r="K21" s="70">
+      <c r="K21" s="69">
         <v>1</v>
       </c>
-      <c r="L21" s="70">
+      <c r="L21" s="69">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M21" s="71">
+      <c r="M21" s="70">
         <v>50</v>
       </c>
-      <c r="N21" s="61" t="s">
+      <c r="N21" s="60" t="s">
         <v>136</v>
       </c>
-      <c r="O21" s="53">
+      <c r="O21" s="52">
         <v>4.3E-3</v>
       </c>
-      <c r="P21" s="76">
+      <c r="P21" s="75">
         <f t="shared" si="2"/>
         <v>0.215</v>
       </c>
@@ -2543,47 +2542,47 @@
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="68" t="s">
+      <c r="C22" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="D22" s="68" t="s">
+      <c r="D22" s="67" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="68" t="s">
+      <c r="E22" s="67" t="s">
         <v>68</v>
       </c>
-      <c r="F22" s="69" t="s">
+      <c r="F22" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="G22" s="68" t="s">
+      <c r="G22" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H22" s="69" t="s">
+      <c r="H22" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="I22" s="68" t="s">
+      <c r="I22" s="67" t="s">
         <v>148</v>
       </c>
-      <c r="J22" s="69" t="s">
+      <c r="J22" s="68" t="s">
         <v>116</v>
       </c>
-      <c r="K22" s="68">
+      <c r="K22" s="67">
         <v>1</v>
       </c>
-      <c r="L22" s="68">
+      <c r="L22" s="67">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M22" s="69">
+      <c r="M22" s="68">
         <v>100</v>
       </c>
-      <c r="N22" s="58" t="s">
+      <c r="N22" s="57" t="s">
         <v>136</v>
       </c>
-      <c r="O22" s="51">
+      <c r="O22" s="50">
         <v>1.5E-3</v>
       </c>
-      <c r="P22" s="75">
+      <c r="P22" s="74">
         <f t="shared" si="2"/>
         <v>0.15</v>
       </c>
@@ -2595,47 +2594,47 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="70" t="s">
+      <c r="C23" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="70" t="s">
+      <c r="D23" s="69" t="s">
         <v>48</v>
       </c>
-      <c r="E23" s="70" t="s">
+      <c r="E23" s="69" t="s">
         <v>69</v>
       </c>
-      <c r="F23" s="71" t="s">
+      <c r="F23" s="70" t="s">
         <v>83</v>
       </c>
-      <c r="G23" s="70" t="s">
+      <c r="G23" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H23" s="71" t="s">
+      <c r="H23" s="70" t="s">
         <v>92</v>
       </c>
-      <c r="I23" s="70" t="s">
+      <c r="I23" s="69" t="s">
         <v>149</v>
       </c>
-      <c r="J23" s="71" t="s">
+      <c r="J23" s="70" t="s">
         <v>117</v>
       </c>
-      <c r="K23" s="70">
+      <c r="K23" s="69">
         <v>4</v>
       </c>
-      <c r="L23" s="70">
+      <c r="L23" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="M23" s="71">
+      <c r="M23" s="70">
         <v>100</v>
       </c>
-      <c r="N23" s="59" t="s">
+      <c r="N23" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="O23" s="50">
+      <c r="O23" s="49">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="P23" s="76">
+      <c r="P23" s="75">
         <f t="shared" si="2"/>
         <v>0.12</v>
       </c>
@@ -2647,47 +2646,47 @@
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="68" t="s">
+      <c r="C24" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="68" t="s">
+      <c r="D24" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="68" t="s">
+      <c r="E24" s="67" t="s">
         <v>68</v>
       </c>
-      <c r="F24" s="69" t="s">
+      <c r="F24" s="68" t="s">
         <v>84</v>
       </c>
-      <c r="G24" s="68" t="s">
+      <c r="G24" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H24" s="69" t="s">
+      <c r="H24" s="68" t="s">
         <v>99</v>
       </c>
-      <c r="I24" s="68" t="s">
+      <c r="I24" s="67" t="s">
         <v>150</v>
       </c>
-      <c r="J24" s="69" t="s">
+      <c r="J24" s="68" t="s">
         <v>118</v>
       </c>
-      <c r="K24" s="68">
+      <c r="K24" s="67">
         <v>5</v>
       </c>
-      <c r="L24" s="68">
+      <c r="L24" s="67">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="M24" s="69">
+      <c r="M24" s="68">
         <v>100</v>
       </c>
-      <c r="N24" s="58" t="s">
+      <c r="N24" s="57" t="s">
         <v>136</v>
       </c>
-      <c r="O24" s="51">
+      <c r="O24" s="50">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="P24" s="75">
+      <c r="P24" s="74">
         <f t="shared" si="2"/>
         <v>0.16999999999999998</v>
       </c>
@@ -2699,47 +2698,47 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="70" t="s">
+      <c r="C25" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="70" t="s">
+      <c r="D25" s="69" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="70" t="s">
+      <c r="E25" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="F25" s="71" t="s">
+      <c r="F25" s="70" t="s">
         <v>85</v>
       </c>
-      <c r="G25" s="70" t="s">
+      <c r="G25" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H25" s="71" t="s">
+      <c r="H25" s="70" t="s">
         <v>92</v>
       </c>
-      <c r="I25" s="70" t="s">
+      <c r="I25" s="69" t="s">
         <v>151</v>
       </c>
-      <c r="J25" s="71" t="s">
+      <c r="J25" s="70" t="s">
         <v>119</v>
       </c>
-      <c r="K25" s="70">
+      <c r="K25" s="69">
         <v>5</v>
       </c>
-      <c r="L25" s="70">
+      <c r="L25" s="69">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="M25" s="71">
+      <c r="M25" s="70">
         <v>50</v>
       </c>
-      <c r="N25" s="59" t="s">
+      <c r="N25" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="O25" s="50">
+      <c r="O25" s="49">
         <v>1.52E-2</v>
       </c>
-      <c r="P25" s="76">
+      <c r="P25" s="75">
         <f t="shared" si="2"/>
         <v>0.76</v>
       </c>
@@ -2751,47 +2750,47 @@
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="68" t="s">
+      <c r="C26" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="68" t="s">
+      <c r="D26" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="E26" s="68" t="s">
+      <c r="E26" s="67" t="s">
         <v>68</v>
       </c>
-      <c r="F26" s="69" t="s">
+      <c r="F26" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="G26" s="68" t="s">
+      <c r="G26" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H26" s="69" t="s">
+      <c r="H26" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="I26" s="68" t="s">
+      <c r="I26" s="67" t="s">
         <v>152</v>
       </c>
-      <c r="J26" s="69" t="s">
+      <c r="J26" s="68" t="s">
         <v>120</v>
       </c>
-      <c r="K26" s="68">
+      <c r="K26" s="67">
         <v>1</v>
       </c>
-      <c r="L26" s="68">
+      <c r="L26" s="67">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M26" s="69">
+      <c r="M26" s="68">
         <v>100</v>
       </c>
-      <c r="N26" s="58" t="s">
+      <c r="N26" s="57" t="s">
         <v>136</v>
       </c>
-      <c r="O26" s="51">
+      <c r="O26" s="50">
         <v>1.5E-3</v>
       </c>
-      <c r="P26" s="75">
+      <c r="P26" s="74">
         <f t="shared" si="2"/>
         <v>0.15</v>
       </c>
@@ -2803,47 +2802,47 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="70" t="s">
+      <c r="C27" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="70" t="s">
+      <c r="D27" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="70" t="s">
+      <c r="E27" s="69" t="s">
         <v>68</v>
       </c>
-      <c r="F27" s="71" t="s">
+      <c r="F27" s="70" t="s">
         <v>154</v>
       </c>
-      <c r="G27" s="70" t="s">
+      <c r="G27" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H27" s="71" t="s">
+      <c r="H27" s="70" t="s">
         <v>100</v>
       </c>
-      <c r="I27" s="70" t="s">
+      <c r="I27" s="69" t="s">
         <v>153</v>
       </c>
-      <c r="J27" s="71" t="s">
+      <c r="J27" s="70" t="s">
         <v>121</v>
       </c>
-      <c r="K27" s="70">
+      <c r="K27" s="69">
         <v>1</v>
       </c>
-      <c r="L27" s="70">
+      <c r="L27" s="69">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M27" s="71">
+      <c r="M27" s="70">
         <v>100</v>
       </c>
-      <c r="N27" s="63" t="s">
+      <c r="N27" s="62" t="s">
         <v>136</v>
       </c>
-      <c r="O27" s="54">
+      <c r="O27" s="53">
         <v>1.4E-3</v>
       </c>
-      <c r="P27" s="76">
+      <c r="P27" s="75">
         <f t="shared" si="2"/>
         <v>0.13999999999999999</v>
       </c>
@@ -2855,47 +2854,47 @@
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="68" t="s">
+      <c r="C28" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="68" t="s">
+      <c r="D28" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="E28" s="68" t="s">
+      <c r="E28" s="67" t="s">
         <v>125</v>
       </c>
-      <c r="F28" s="69" t="s">
+      <c r="F28" s="68" t="s">
         <v>70</v>
       </c>
-      <c r="G28" s="68" t="s">
+      <c r="G28" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H28" s="69" t="s">
+      <c r="H28" s="68" t="s">
         <v>101</v>
       </c>
-      <c r="I28" s="68" t="s">
+      <c r="I28" s="67" t="s">
         <v>156</v>
       </c>
-      <c r="J28" s="69" t="s">
+      <c r="J28" s="68" t="s">
         <v>139</v>
       </c>
-      <c r="K28" s="68">
+      <c r="K28" s="67">
         <v>1</v>
       </c>
-      <c r="L28" s="68">
+      <c r="L28" s="67">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M28" s="69">
+      <c r="M28" s="68">
         <v>10</v>
       </c>
-      <c r="N28" s="62" t="s">
+      <c r="N28" s="61" t="s">
         <v>136</v>
       </c>
-      <c r="O28" s="55">
+      <c r="O28" s="54">
         <v>5.9499999999999997E-2</v>
       </c>
-      <c r="P28" s="77">
+      <c r="P28" s="76">
         <f t="shared" si="2"/>
         <v>0.59499999999999997</v>
       </c>
@@ -2907,47 +2906,47 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="70" t="s">
+      <c r="C29" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="D29" s="70" t="s">
+      <c r="D29" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="E29" s="70" t="s">
+      <c r="E29" s="69" t="s">
         <v>71</v>
       </c>
-      <c r="F29" s="71" t="s">
+      <c r="F29" s="70" t="s">
         <v>87</v>
       </c>
-      <c r="G29" s="70" t="s">
+      <c r="G29" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H29" s="71" t="s">
+      <c r="H29" s="70" t="s">
         <v>102</v>
       </c>
-      <c r="I29" s="70" t="s">
+      <c r="I29" s="69" t="s">
         <v>157</v>
       </c>
-      <c r="J29" s="71" t="s">
+      <c r="J29" s="70" t="s">
         <v>139</v>
       </c>
-      <c r="K29" s="70">
+      <c r="K29" s="69">
         <v>1</v>
       </c>
-      <c r="L29" s="70">
+      <c r="L29" s="69">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M29" s="71">
+      <c r="M29" s="70">
         <v>7</v>
       </c>
-      <c r="N29" s="59" t="s">
+      <c r="N29" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="O29" s="50">
+      <c r="O29" s="49">
         <v>0.4869</v>
       </c>
-      <c r="P29" s="78">
+      <c r="P29" s="77">
         <f t="shared" si="2"/>
         <v>3.4083000000000001</v>
       </c>
@@ -2959,47 +2958,47 @@
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="68" t="s">
+      <c r="C30" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="68" t="s">
+      <c r="D30" s="67" t="s">
         <v>55</v>
       </c>
-      <c r="E30" s="68" t="s">
+      <c r="E30" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="F30" s="69" t="s">
+      <c r="F30" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="G30" s="68" t="s">
+      <c r="G30" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="H30" s="69" t="s">
+      <c r="H30" s="68" t="s">
         <v>103</v>
       </c>
-      <c r="I30" s="68" t="s">
+      <c r="I30" s="67" t="s">
         <v>158</v>
       </c>
-      <c r="J30" s="69" t="s">
+      <c r="J30" s="68" t="s">
         <v>139</v>
       </c>
-      <c r="K30" s="68">
+      <c r="K30" s="67">
         <v>1</v>
       </c>
-      <c r="L30" s="68">
+      <c r="L30" s="67">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M30" s="69">
+      <c r="M30" s="68">
         <v>7</v>
       </c>
-      <c r="N30" s="58" t="s">
+      <c r="N30" s="57" t="s">
         <v>136</v>
       </c>
-      <c r="O30" s="51">
+      <c r="O30" s="50">
         <v>1.8827</v>
       </c>
-      <c r="P30" s="75">
+      <c r="P30" s="74">
         <f t="shared" si="2"/>
         <v>13.178900000000001</v>
       </c>
@@ -3011,47 +3010,47 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="70" t="s">
+      <c r="C31" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="D31" s="70" t="s">
+      <c r="D31" s="69" t="s">
         <v>56</v>
       </c>
-      <c r="E31" s="70" t="s">
+      <c r="E31" s="69" t="s">
         <v>164</v>
       </c>
-      <c r="F31" s="71" t="s">
+      <c r="F31" s="70" t="s">
         <v>73</v>
       </c>
-      <c r="G31" s="70" t="s">
+      <c r="G31" s="69" t="s">
         <v>161</v>
       </c>
-      <c r="H31" s="71" t="s">
+      <c r="H31" s="70" t="s">
         <v>104</v>
       </c>
-      <c r="I31" s="70" t="s">
+      <c r="I31" s="69" t="s">
         <v>159</v>
       </c>
-      <c r="J31" s="71" t="s">
+      <c r="J31" s="70" t="s">
         <v>139</v>
       </c>
-      <c r="K31" s="70">
+      <c r="K31" s="69">
         <v>1</v>
       </c>
-      <c r="L31" s="70">
+      <c r="L31" s="69">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M31" s="71">
+      <c r="M31" s="70">
         <v>7</v>
       </c>
-      <c r="N31" s="59" t="s">
+      <c r="N31" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="O31" s="50">
+      <c r="O31" s="49">
         <v>0.95220000000000005</v>
       </c>
-      <c r="P31" s="76">
+      <c r="P31" s="75">
         <f t="shared" si="2"/>
         <v>6.6654</v>
       </c>
@@ -3063,51 +3062,51 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="72" t="s">
+      <c r="C32" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="D32" s="72" t="s">
+      <c r="D32" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E32" s="72" t="s">
+      <c r="E32" s="71" t="s">
         <v>165</v>
       </c>
-      <c r="F32" s="73" t="s">
+      <c r="F32" s="72" t="s">
         <v>74</v>
       </c>
-      <c r="G32" s="72" t="s">
+      <c r="G32" s="71" t="s">
         <v>161</v>
       </c>
-      <c r="H32" s="73" t="s">
+      <c r="H32" s="72" t="s">
         <v>105</v>
       </c>
-      <c r="I32" s="72" t="s">
+      <c r="I32" s="71" t="s">
         <v>160</v>
       </c>
-      <c r="J32" s="73" t="s">
+      <c r="J32" s="72" t="s">
         <v>139</v>
       </c>
-      <c r="K32" s="72">
+      <c r="K32" s="71">
         <v>1</v>
       </c>
-      <c r="L32" s="72">
+      <c r="L32" s="71">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M32" s="73">
+      <c r="M32" s="72">
         <v>7</v>
       </c>
-      <c r="N32" s="64" t="s">
+      <c r="N32" s="63" t="s">
         <v>136</v>
       </c>
-      <c r="O32" s="66">
+      <c r="O32" s="65">
         <v>0.54279999999999995</v>
       </c>
-      <c r="P32" s="79">
+      <c r="P32" s="78">
         <f t="shared" si="2"/>
         <v>3.7995999999999999</v>
       </c>
-      <c r="Q32" s="67"/>
+      <c r="Q32" s="66"/>
     </row>
     <row r="33" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -3124,16 +3123,16 @@
       <c r="J33" s="29"/>
       <c r="K33" s="29"/>
       <c r="L33" s="43"/>
-      <c r="M33" s="86" t="s">
+      <c r="M33" s="85" t="s">
         <v>162</v>
       </c>
-      <c r="N33" s="87"/>
-      <c r="O33" s="87"/>
-      <c r="P33" s="74">
+      <c r="N33" s="86"/>
+      <c r="O33" s="86"/>
+      <c r="P33" s="73">
         <f>SUM(P10:P32)</f>
         <v>56.282599999999995</v>
       </c>
-      <c r="Q33" s="65"/>
+      <c r="Q33" s="64"/>
     </row>
     <row r="34" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
@@ -3150,12 +3149,15 @@
       <c r="J34" s="9"/>
       <c r="K34" s="9"/>
       <c r="L34" s="42"/>
-      <c r="M34" s="80" t="s">
+      <c r="M34" s="79" t="s">
         <v>163</v>
       </c>
-      <c r="N34" s="81"/>
-      <c r="O34" s="81"/>
-      <c r="P34" s="47"/>
+      <c r="N34" s="80"/>
+      <c r="O34" s="80"/>
+      <c r="P34" s="89">
+        <f>P33/5</f>
+        <v>11.256519999999998</v>
+      </c>
       <c r="Q34" s="31"/>
     </row>
   </sheetData>
@@ -3167,29 +3169,29 @@
     <mergeCell ref="J1:L1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="N10" r:id="rId1" xr:uid="{7D1D9C0C-E083-4202-8537-45FC2922DBEF}"/>
-    <hyperlink ref="N11" r:id="rId2" xr:uid="{BF6D986C-36B1-47BD-A90A-69766656A3E2}"/>
-    <hyperlink ref="N12" r:id="rId3" xr:uid="{77ABCD45-E4E8-4D73-AFA8-265A1929B1FC}"/>
-    <hyperlink ref="N13" r:id="rId4" xr:uid="{6ADB7F75-3CAA-4B0A-B9BC-137A9FCD0C11}"/>
-    <hyperlink ref="N14" r:id="rId5" xr:uid="{2C2EB80B-FD50-4F70-8159-BA69500B8357}"/>
-    <hyperlink ref="N15" r:id="rId6" xr:uid="{E0307834-10EF-499E-8B8C-008CD18AD267}"/>
-    <hyperlink ref="N16" r:id="rId7" xr:uid="{1D4B5633-3344-4F0D-96C8-E6943B9D46F5}"/>
-    <hyperlink ref="N17" r:id="rId8" xr:uid="{A2980A0C-A0AC-4E2B-AFA4-78736A9F5A0D}"/>
-    <hyperlink ref="N18" r:id="rId9" xr:uid="{4DF83AAC-A88A-4CDF-8AE2-2CD019DAB87E}"/>
-    <hyperlink ref="N19" r:id="rId10" xr:uid="{A4669AA6-4D51-4B94-A266-EBBFC0346D9E}"/>
-    <hyperlink ref="N20" r:id="rId11" xr:uid="{49BF3C61-D3A2-4088-846D-08620D777F72}"/>
-    <hyperlink ref="N21" r:id="rId12" xr:uid="{6C26B9A4-5A30-46CC-9E33-3C5A9E6C979A}"/>
-    <hyperlink ref="N22" r:id="rId13" xr:uid="{75308361-4DA2-458E-BB7A-B3E632E3E180}"/>
-    <hyperlink ref="N23" r:id="rId14" xr:uid="{E6F22E7C-F575-402A-97EC-E8F62CF9EE7D}"/>
-    <hyperlink ref="N24" r:id="rId15" xr:uid="{9AB8D03C-D60C-4639-8093-13E63E8C09F8}"/>
-    <hyperlink ref="N25" r:id="rId16" xr:uid="{94E5EA2A-014A-4092-83C5-FAF4E83F71FD}"/>
-    <hyperlink ref="N26" r:id="rId17" xr:uid="{E2B1E76C-4B6B-4676-8A54-5FD51D959CD8}"/>
-    <hyperlink ref="N27" r:id="rId18" xr:uid="{2698B370-BBA7-4FA7-A624-F369F7099ED1}"/>
-    <hyperlink ref="N28" r:id="rId19" xr:uid="{B743A9F0-C548-4311-B352-A40E5C2B0A7D}"/>
-    <hyperlink ref="N29" r:id="rId20" xr:uid="{C0A21BFC-A8AF-463A-B15F-00A8E333E505}"/>
-    <hyperlink ref="N30" r:id="rId21" xr:uid="{F718CA87-7FE6-4F67-8ECC-42E6140BA634}"/>
-    <hyperlink ref="N31" r:id="rId22" xr:uid="{FB82703E-54B0-4C79-85D1-A65A59DF7E2C}"/>
-    <hyperlink ref="N32" r:id="rId23" xr:uid="{B394E64C-FBEC-4BE3-AD0B-605A9D6C2257}"/>
+    <hyperlink ref="N10" r:id="rId1"/>
+    <hyperlink ref="N11" r:id="rId2"/>
+    <hyperlink ref="N12" r:id="rId3"/>
+    <hyperlink ref="N13" r:id="rId4"/>
+    <hyperlink ref="N14" r:id="rId5"/>
+    <hyperlink ref="N15" r:id="rId6"/>
+    <hyperlink ref="N16" r:id="rId7"/>
+    <hyperlink ref="N17" r:id="rId8"/>
+    <hyperlink ref="N18" r:id="rId9"/>
+    <hyperlink ref="N19" r:id="rId10"/>
+    <hyperlink ref="N20" r:id="rId11"/>
+    <hyperlink ref="N21" r:id="rId12"/>
+    <hyperlink ref="N22" r:id="rId13"/>
+    <hyperlink ref="N23" r:id="rId14"/>
+    <hyperlink ref="N24" r:id="rId15"/>
+    <hyperlink ref="N25" r:id="rId16"/>
+    <hyperlink ref="N26" r:id="rId17"/>
+    <hyperlink ref="N27" r:id="rId18"/>
+    <hyperlink ref="N28" r:id="rId19"/>
+    <hyperlink ref="N29" r:id="rId20"/>
+    <hyperlink ref="N30" r:id="rId21"/>
+    <hyperlink ref="N31" r:id="rId22"/>
+    <hyperlink ref="N32" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId24"/>

</xml_diff>

<commit_message>
per board quantity formatted #14
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/FLST_Client BOM.xlsx
+++ b/Deliverables/BOM/FLST_Client BOM.xlsx
@@ -1095,7 +1095,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1341,7 +1341,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="16" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1679,7 +1682,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -3154,11 +3157,17 @@
       </c>
       <c r="N34" s="80"/>
       <c r="O34" s="80"/>
-      <c r="P34" s="89">
+      <c r="P34" s="90">
         <f>P33/5</f>
         <v>11.256519999999998</v>
       </c>
       <c r="Q34" s="31"/>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="P38" s="89">
+        <f>P33*2</f>
+        <v>112.56519999999999</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>